<commit_message>
Update route 664 schedule to match daily timetable.
Both directions now share the full departure list from the operator schedule.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/schedule-664.xlsx
+++ b/public/schedule-664.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Schedule" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,52 +412,100 @@
         <v>7:00</v>
       </c>
       <c r="B2" t="str">
-        <v>8:15</v>
+        <v>7:00</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>9:30</v>
+        <v>8:15</v>
       </c>
       <c r="B3" t="str">
-        <v>11:00</v>
+        <v>8:15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>12:30</v>
+        <v>9:30</v>
       </c>
       <c r="B4" t="str">
-        <v>14:30</v>
+        <v>9:30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>15:30</v>
+        <v>11:00</v>
       </c>
       <c r="B5" t="str">
-        <v>17:40</v>
+        <v>11:00</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>18:30</v>
+        <v>12:30</v>
       </c>
       <c r="B6" t="str">
-        <v>20:00</v>
+        <v>12:30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>14:30</v>
+      </c>
+      <c r="B7" t="str">
+        <v>14:30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="B8" t="str">
+        <v>15:30</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>17:40</v>
+      </c>
+      <c r="B9" t="str">
+        <v>17:40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="B10" t="str">
+        <v>18:30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="B11" t="str">
+        <v>20:00</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>21:00</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B12" t="str">
+        <v>21:00</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>22:10</v>
+      </c>
+      <c r="B13" t="str">
         <v>22:10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>